<commit_message>
Add Dani portfolio pitch, audited financial model and spatial presentation
</commit_message>
<xml_diff>
--- a/modelo-financeiro.xlsx
+++ b/modelo-financeiro.xlsx
@@ -1,167 +1,226 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia primeiro" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Premissas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infraestrutura" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agenda" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conservador" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expansao" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacidade" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verificado" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sociedade" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fontes" sheetId="12" state="visible" r:id="rId12"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <ns0:workbookPr/>
+  <ns0:workbookProtection/>
+  <ns0:bookViews>
+    <ns0:workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </ns0:bookViews>
+  <ns0:sheets>
+    <ns0:sheet name="Leia primeiro" sheetId="1" state="visible" ns1:id="rId1"/>
+    <ns0:sheet name="Premissas" sheetId="2" state="visible" ns1:id="rId2"/>
+    <ns0:sheet name="Infraestrutura" sheetId="3" state="visible" ns1:id="rId3"/>
+    <ns0:sheet name="Agenda" sheetId="4" state="visible" ns1:id="rId4"/>
+    <ns0:sheet name="Conservador" sheetId="5" state="visible" ns1:id="rId5"/>
+    <ns0:sheet name="Base" sheetId="6" state="visible" ns1:id="rId6"/>
+    <ns0:sheet name="Expansao" sheetId="7" state="visible" ns1:id="rId7"/>
+    <ns0:sheet name="Resumo" sheetId="8" state="visible" ns1:id="rId8"/>
+    <ns0:sheet name="Capacidade" sheetId="9" state="visible" ns1:id="rId9"/>
+    <ns0:sheet name="Verificado" sheetId="10" state="visible" ns1:id="rId10"/>
+    <ns0:sheet name="Sociedade" sheetId="11" state="visible" ns1:id="rId11"/>
+    <ns0:sheet name="Fontes" sheetId="12" state="visible" ns1:id="rId12"/>
+    <ns0:sheet name="Perspectivas" sheetId="13" ns1:id="rId15"/>
+    <ns0:sheet name="Desenvolvimento" sheetId="14" ns1:id="rId16"/>
+    <ns0:sheet name="Monetização" sheetId="15" ns1:id="rId17"/>
+  </ns0:sheets>
+  <ns0:definedNames/>
+  <ns0:calcPr calcId="124519" fullCalcOnLoad="1"/>
+</ns0:workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-  </numFmts>
-  <fonts count="3">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11"/>
-    </font>
-  </fonts>
-  <fills count="3">
-    <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0017352E"/>
-      </patternFill>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-</styleSheet>
+<ns0:styleSheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:numFmts count="4">
+    <ns0:numFmt numFmtId="164" formatCode="0.0%"/>
+    <ns0:numFmt numFmtId="165" formatCode="&quot;R$&quot; #,##0.00;[Red]-&quot;R$&quot; #,##0.00"/>
+    <ns0:numFmt numFmtId="166" formatCode="0.00"/>
+    <ns0:numFmt numFmtId="167" formatCode="0.0%"/>
+  </ns0:numFmts>
+  <ns0:fonts count="5">
+    <ns0:font>
+      <ns0:name val="Calibri"/>
+      <ns0:family val="2"/>
+      <ns0:color theme="1"/>
+      <ns0:sz val="11"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="Calibri"/>
+      <ns0:b val="1"/>
+      <ns0:color rgb="00FFFFFF"/>
+      <ns0:sz val="12"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:name val="Calibri"/>
+      <ns0:sz val="11"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:color theme="1"/>
+      <ns0:name val="Calibri"/>
+      <ns0:family val="2"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FFFFFFFF"/>
+      <ns0:name val="Calibri"/>
+      <ns0:family val="2"/>
+      <ns0:scheme val="minor"/>
+    </ns0:font>
+  </ns0:fonts>
+  <ns0:fills count="6">
+    <ns0:fill>
+      <ns0:patternFill/>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="gray125"/>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="0017352E"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="none"/>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="gray125"/>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FF17352E"/>
+        <ns0:bgColor indexed="64"/>
+      </ns0:patternFill>
+    </ns0:fill>
+  </ns0:fills>
+  <ns0:borders count="2">
+    <ns0:border>
+      <ns0:left/>
+      <ns0:right/>
+      <ns0:top/>
+      <ns0:bottom/>
+      <ns0:diagonal/>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left/>
+      <ns0:right/>
+      <ns0:top/>
+      <ns0:bottom/>
+      <ns0:diagonal/>
+    </ns0:border>
+  </ns0:borders>
+  <ns0:cellStyleXfs count="1">
+    <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </ns0:cellStyleXfs>
+  <ns0:cellXfs count="12">
+    <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <ns0:xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <ns0:alignment vertical="center" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <ns0:alignment vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <ns0:alignment vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <ns0:alignment vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0"/>
+    <ns0:xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <ns0:alignment vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyAlignment="1">
+      <ns0:alignment vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <ns0:alignment vertical="top"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="166" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <ns0:alignment vertical="top"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="1" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <ns0:alignment vertical="top"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="167" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <ns0:alignment vertical="top"/>
+    </ns0:xf>
+  </ns0:cellXfs>
+  <ns0:cellStyles count="1">
+    <ns0:cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </ns0:cellStyles>
+  <ns0:tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <ns0:colors>
+    <ns0:indexedColors>
+      <ns0:rgbColor rgb="00000000"/>
+      <ns0:rgbColor rgb="00FFFFFF"/>
+      <ns0:rgbColor rgb="00FF0000"/>
+      <ns0:rgbColor rgb="0000FF00"/>
+      <ns0:rgbColor rgb="000000FF"/>
+      <ns0:rgbColor rgb="00FFFF00"/>
+      <ns0:rgbColor rgb="00FF00FF"/>
+      <ns0:rgbColor rgb="0000FFFF"/>
+      <ns0:rgbColor rgb="00000000"/>
+      <ns0:rgbColor rgb="00FFFFFF"/>
+      <ns0:rgbColor rgb="00FF0000"/>
+      <ns0:rgbColor rgb="0000FF00"/>
+      <ns0:rgbColor rgb="000000FF"/>
+      <ns0:rgbColor rgb="00FFFF00"/>
+      <ns0:rgbColor rgb="00FF00FF"/>
+      <ns0:rgbColor rgb="0000FFFF"/>
+      <ns0:rgbColor rgb="00800000"/>
+      <ns0:rgbColor rgb="00008000"/>
+      <ns0:rgbColor rgb="00000080"/>
+      <ns0:rgbColor rgb="00808000"/>
+      <ns0:rgbColor rgb="00800080"/>
+      <ns0:rgbColor rgb="00008080"/>
+      <ns0:rgbColor rgb="00C0C0C0"/>
+      <ns0:rgbColor rgb="00808080"/>
+      <ns0:rgbColor rgb="009999FF"/>
+      <ns0:rgbColor rgb="00993366"/>
+      <ns0:rgbColor rgb="00FFFFCC"/>
+      <ns0:rgbColor rgb="00CCFFFF"/>
+      <ns0:rgbColor rgb="00660066"/>
+      <ns0:rgbColor rgb="00FF8080"/>
+      <ns0:rgbColor rgb="000066CC"/>
+      <ns0:rgbColor rgb="00CCCCFF"/>
+      <ns0:rgbColor rgb="00000080"/>
+      <ns0:rgbColor rgb="00FF00FF"/>
+      <ns0:rgbColor rgb="00FFFF00"/>
+      <ns0:rgbColor rgb="0000FFFF"/>
+      <ns0:rgbColor rgb="00800080"/>
+      <ns0:rgbColor rgb="00800000"/>
+      <ns0:rgbColor rgb="00008080"/>
+      <ns0:rgbColor rgb="000000FF"/>
+      <ns0:rgbColor rgb="0000CCFF"/>
+      <ns0:rgbColor rgb="00CCFFFF"/>
+      <ns0:rgbColor rgb="00CCFFCC"/>
+      <ns0:rgbColor rgb="00FFFF99"/>
+      <ns0:rgbColor rgb="0099CCFF"/>
+      <ns0:rgbColor rgb="00FF99CC"/>
+      <ns0:rgbColor rgb="00CC99FF"/>
+      <ns0:rgbColor rgb="00FFCC99"/>
+      <ns0:rgbColor rgb="003366FF"/>
+      <ns0:rgbColor rgb="0033CCCC"/>
+      <ns0:rgbColor rgb="0099CC00"/>
+      <ns0:rgbColor rgb="00FFCC00"/>
+      <ns0:rgbColor rgb="00FF9900"/>
+      <ns0:rgbColor rgb="00FF6600"/>
+      <ns0:rgbColor rgb="00666699"/>
+      <ns0:rgbColor rgb="00969696"/>
+      <ns0:rgbColor rgb="00003366"/>
+      <ns0:rgbColor rgb="00339966"/>
+      <ns0:rgbColor rgb="00003300"/>
+      <ns0:rgbColor rgb="00333300"/>
+      <ns0:rgbColor rgb="00993300"/>
+      <ns0:rgbColor rgb="00993366"/>
+      <ns0:rgbColor rgb="00333399"/>
+      <ns0:rgbColor rgb="00333333"/>
+    </ns0:indexedColors>
+  </ns0:colors>
+</ns0:styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7269,6 +7328,1500 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetPr>
+    <ns0:pageSetUpPr fitToPage="1"/>
+  </ns0:sheetPr>
+  <ns0:dimension ref="A1:E23"/>
+  <ns0:sheetFormatPr defaultRowHeight="15"/>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="43.7109375" customWidth="1"/>
+    <ns0:col min="2" max="4" width="22.7109375" customWidth="1"/>
+    <ns0:col min="5" max="5" width="95.7109375" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" ht="42" customHeight="1">
+      <ns0:c r="A1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Item / alcance</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Capital R$100 mil</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Capital R$150 mil</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Capital R$200 mil</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Fonte / leitura</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2" ht="46" customHeight="1">
+      <ns0:c r="A2" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Capital total inicial</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B2" s="8">
+        <ns0:v>100000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C2" s="8">
+        <ns0:v>150000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D2" s="8">
+        <ns0:v>200000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E2" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hipóteses de capital; não preço ao cliente nem autorização de compra</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3" ht="46" customHeight="1">
+      <ns0:c r="A3" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Equipamentos</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3" s="8">
+        <ns0:f>Premissas!$B$21</ns0:f>
+        <ns0:v>76000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C3" s="8">
+        <ns0:f>Premissas!$B$21</ns0:f>
+        <ns0:v>76000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D3" s="8">
+        <ns0:f>Premissas!$B$21</ns0:f>
+        <ns0:v>76000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E3" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hardware R$76 mil; uma DGX em todas as perspectivas</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4" ht="46" customHeight="1">
+      <ns0:c r="A4" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Pré-operacional</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B4" s="8">
+        <ns0:f>Premissas!$B$22</ns0:f>
+        <ns0:v>24000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C4" s="8">
+        <ns0:f>Premissas!$B$22</ns0:f>
+        <ns0:v>24000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D4" s="8">
+        <ns0:f>Premissas!$B$22</ns0:f>
+        <ns0:v>24000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E4" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Jurídico R$12 mil + segurança R$12 mil; hipóteses</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5" ht="46" customHeight="1">
+      <ns0:c r="A5" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>M0: desembolso inicial</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" s="8">
+        <ns0:f>SUM(B3:B4)</ns0:f>
+        <ns0:v>100000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C5" s="8">
+        <ns0:f>SUM(C3:C4)</ns0:f>
+        <ns0:v>100000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D5" s="8">
+        <ns0:f>SUM(D3:D4)</ns0:f>
+        <ns0:v>100000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E5" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Equipamentos + preparação, sem operação mensal</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6" ht="46" customHeight="1">
+      <ns0:c r="A6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Fixo mensal inicial</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B6" s="8">
+        <ns0:f>Premissas!$B$10</ns0:f>
+        <ns0:v>37000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C6" s="8">
+        <ns0:f>Premissas!$B$10</ns0:f>
+        <ns0:v>37000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D6" s="8">
+        <ns0:f>Premissas!$B$10</ns0:f>
+        <ns0:v>37000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Meses 1–12; R$37 mil; pessoas de P&amp;D não são implantação</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7" ht="46" customHeight="1">
+      <ns0:c r="A7" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Caixa após M0</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B7" s="8">
+        <ns0:f>B2-B5</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="C7" s="8">
+        <ns0:f>C2-C5</ns0:f>
+        <ns0:v>50000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D7" s="8">
+        <ns0:f>D2-D5</ns0:f>
+        <ns0:v>100000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E7" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Capital − M0; sem receita nem reserva</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8" ht="46" customHeight="1">
+      <ns0:c r="A8" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Meses aritméticos financiados</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B8" s="9">
+        <ns0:f>MAX(0,B7/B6)</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="C8" s="9">
+        <ns0:f>MAX(0,C7/C6)</ns0:f>
+        <ns0:v>1.3513513513513513</ns0:v>
+      </ns0:c>
+      <ns0:c r="D8" s="9">
+        <ns0:f>MAX(0,D7/D6)</ns0:f>
+        <ns0:v>2.7027027027027026</ns0:v>
+      </ns0:c>
+      <ns0:c r="E8" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Não representa parcelamento de despesas ou garantia de desenvolvimento</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9" ht="46" customHeight="1">
+      <ns0:c r="A9" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Meses completos financiados</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B9" s="10">
+        <ns0:f>INT(B8)</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="C9" s="10">
+        <ns0:f>INT(C8)</ns0:f>
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="D9" s="10">
+        <ns0:f>INT(D8)</ns0:f>
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="E9" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Parte inteira do prazo; sem reduzir fixos</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="10" ht="46" customHeight="1">
+      <ns0:c r="A10" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Saldo após meses completos</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B10" s="8">
+        <ns0:f>B7-B9*B6</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="C10" s="8">
+        <ns0:f>C7-C9*C6</ns0:f>
+        <ns0:v>13000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D10" s="8">
+        <ns0:f>D7-D9*D6</ns0:f>
+        <ns0:v>26000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E10" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Insuficiente para financiar integralmente o mês seguinte</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="11" ht="46" customHeight="1">
+      <ns0:c r="A11" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>M0 + três meses</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B11" s="8">
+        <ns0:f>B5+3*B6</ns0:f>
+        <ns0:v>211000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C11" s="8">
+        <ns0:f>C5+3*C6</ns0:f>
+        <ns0:v>211000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D11" s="8">
+        <ns0:f>D5+3*D6</ns0:f>
+        <ns0:v>211000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E11" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Sem reserva, receita ou custos de entrega</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="12" ht="46" customHeight="1">
+      <ns0:c r="A12" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Falta para três meses</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B12" s="8">
+        <ns0:f>MAX(0,B11-B2)</ns0:f>
+        <ns0:v>111000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C12" s="8">
+        <ns0:f>MAX(0,C11-C2)</ns0:f>
+        <ns0:v>61000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D12" s="8">
+        <ns0:f>MAX(0,D11-D2)</ns0:f>
+        <ns0:v>11000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E12" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Capital adicional necessário até o patamar, não garantia de aceite</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="13" ht="46" customHeight="1">
+      <ns0:c r="A13" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>M0 + seis meses</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B13" s="8">
+        <ns0:f>B5+6*B6</ns0:f>
+        <ns0:v>322000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C13" s="8">
+        <ns0:f>C5+6*C6</ns0:f>
+        <ns0:v>322000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D13" s="8">
+        <ns0:f>D5+6*D6</ns0:f>
+        <ns0:v>322000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E13" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Sem reserva, receita ou custos de entrega</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="14" ht="46" customHeight="1">
+      <ns0:c r="A14" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Falta para seis meses</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B14" s="8">
+        <ns0:f>MAX(0,B13-B2)</ns0:f>
+        <ns0:v>222000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C14" s="8">
+        <ns0:f>MAX(0,C13-C2)</ns0:f>
+        <ns0:v>172000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D14" s="8">
+        <ns0:f>MAX(0,D13-D2)</ns0:f>
+        <ns0:v>122000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E14" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>M7 primeira venda-base não comprovada</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="15" ht="46" customHeight="1">
+      <ns0:c r="A15" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Capital-base 24 meses</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B15" s="8">
+        <ns0:f>Resumo!$L$3</ns0:f>
+        <ns0:v>830000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C15" s="8">
+        <ns0:f>Resumo!$L$3</ns0:f>
+        <ns0:v>830000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D15" s="8">
+        <ns0:f>Resumo!$L$3</ns0:f>
+        <ns0:v>830000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E15" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Fluxo com vendas hipotéticas, custos diretos, fixos e reserva; inalterado</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="16" ht="46" customHeight="1">
+      <ns0:c r="A16" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Falta para capital-base 24 meses</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B16" s="8">
+        <ns0:f>MAX(0,B15-B2)</ns0:f>
+        <ns0:v>730000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C16" s="8">
+        <ns0:f>MAX(0,C15-C2)</ns0:f>
+        <ns0:v>680000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D16" s="8">
+        <ns0:f>MAX(0,D15-D2)</ns0:f>
+        <ns0:v>630000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E16" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Diferença entre R$830 mil de planejamento e capital inicial</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="17" ht="46" customHeight="1">
+      <ns0:c r="A17" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Lançamento integral financiado</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B17" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Não</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C17" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Não</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D17" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Não</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E17" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Nenhum capital financia sequer M0 + três meses integralmente</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="18" ht="46" customHeight="1">
+      <ns0:c r="A18" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Infraestrutura do primeiro ano</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B18" s="8">
+        <ns0:f>Infraestrutura!$D$11</ns0:f>
+        <ns0:v>100000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C18" s="8">
+        <ns0:f>Infraestrutura!$D$11</ns0:f>
+        <ns0:v>100000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D18" s="8">
+        <ns0:f>Infraestrutura!$D$11</ns0:f>
+        <ns0:v>100000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E18" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Outra composição: hardware76 + serviços18 + reserva6; não somar novamente</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="19" ht="46" customHeight="1">
+      <ns0:c r="A19" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Preço de implantação do cliente</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B19" s="8">
+        <ns0:f>Premissas!$B$2</ns0:f>
+        <ns0:v>200000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C19" s="8">
+        <ns0:f>Premissas!$B$2</ns0:f>
+        <ns0:v>200000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D19" s="8">
+        <ns0:f>Premissas!$B$2</ns0:f>
+        <ns0:v>200000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E19" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Oferta principal; não aporte ou lucro</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="20" ht="46" customHeight="1">
+      <ns0:c r="A20" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Mensalidade do cliente</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B20" s="8">
+        <ns0:f>Premissas!$B$3</ns0:f>
+        <ns0:v>12000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C20" s="8">
+        <ns0:f>Premissas!$B$3</ns0:f>
+        <ns0:v>12000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D20" s="8">
+        <ns0:f>Premissas!$B$3</ns0:f>
+        <ns0:v>12000</ns0:v>
+      </ns0:c>
+      <ns0:c r="E20" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Após aceite; hipótese comercial, não receita garantida</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="23" ht="72" customHeight="1">
+      <ns0:c r="A23" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Fonte e atualização</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E23" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>planning.json, Premissas, Infraestrutura e Resumo. Entradas B2:D2 editáveis. Fórmulas com cache inicial; recalcular no Excel/LibreOffice ao editar. Textos/CSV são snapshots.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ns0:pageSetup fitToHeight="0" orientation="landscape"/>
+</ns0:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetPr>
+    <ns0:pageSetUpPr fitToPage="1"/>
+  </ns0:sheetPr>
+  <ns0:dimension ref="A1:I13"/>
+  <ns0:sheetFormatPr defaultRowHeight="15"/>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="26.7109375" customWidth="1"/>
+    <ns0:col min="2" max="2" width="42.7109375" customWidth="1"/>
+    <ns0:col min="3" max="3" width="90.7109375" customWidth="1"/>
+    <ns0:col min="4" max="4" width="17.7109375" customWidth="1"/>
+    <ns0:col min="5" max="8" width="23.7109375" customWidth="1"/>
+    <ns0:col min="9" max="9" width="90.7109375" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" ht="42" customHeight="1">
+      <ns0:c r="A1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Período</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Objetivo</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Aceite necessário (não garantia)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Meses acumulados</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>M0 + fixos mínimos</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Falta: 100 mil</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Falta: 150 mil</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Falta: 200 mil</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Condição / fonte</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2" ht="120" customHeight="1">
+      <ns0:c r="A2" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Antes do desembolso</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B2" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Confirmar caixa, comprador-alvo e cotação</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C2" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Cotação brasileira completa, origem do capital, contrato societário, escopo e condições de parada; sem compra automática.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D2" s="10">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="E2" s="8">
+        <ns0:f>Perspectivas!$B$5+D2*Premissas!$B$10</ns0:f>
+        <ns0:v>100000</ns0:v>
+      </ns0:c>
+      <ns0:c r="F2" s="8">
+        <ns0:f>MAX(0,E2-Perspectivas!$B$2)</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="G2" s="8">
+        <ns0:f>MAX(0,E2-Perspectivas!$C$2)</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="H2" s="8">
+        <ns0:f>MAX(0,E2-Perspectivas!$D$2)</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I2" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>planning.json; mínimo financeiro sem reserva, receita e custos de implantação. Antes do desembolso, resolver financiamento. Nos demais marcos, caixa não comprova aceite; parar se faltar acesso, recursos ou segurança.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3" ht="120" customHeight="1">
+      <ns0:c r="A3" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Mês 1</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Transformar a demonstração em núcleo persistente</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C3" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Modelo versionado, identidade, fontes autorizadas e restauração demonstrada. Não equivale a produto comercial homologado.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D3" s="10">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="E3" s="8">
+        <ns0:f>Perspectivas!$B$5+D3*Premissas!$B$10</ns0:f>
+        <ns0:v>137000</ns0:v>
+      </ns0:c>
+      <ns0:c r="F3" s="8">
+        <ns0:f>MAX(0,E3-Perspectivas!$B$2)</ns0:f>
+        <ns0:v>37000</ns0:v>
+      </ns0:c>
+      <ns0:c r="G3" s="8">
+        <ns0:f>MAX(0,E3-Perspectivas!$C$2)</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="H3" s="8">
+        <ns0:f>MAX(0,E3-Perspectivas!$D$2)</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I3" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>planning.json; mínimo financeiro sem reserva, receita e custos de implantação. Antes do desembolso, resolver financiamento. Nos demais marcos, caixa não comprova aceite; parar se faltar acesso, recursos ou segurança.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4" ht="120" customHeight="1">
+      <ns0:c r="A4" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Mês 2</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B4" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Conectar contexto e testar fronteiras</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C4" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Ingestão de fontes de ensaio, consultas com evidência e testes de permissão. Dois conectores de produção ainda dependem de acesso e homologação.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D4" s="10">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="E4" s="8">
+        <ns0:f>Perspectivas!$B$5+D4*Premissas!$B$10</ns0:f>
+        <ns0:v>174000</ns0:v>
+      </ns0:c>
+      <ns0:c r="F4" s="8">
+        <ns0:f>MAX(0,E4-Perspectivas!$B$2)</ns0:f>
+        <ns0:v>74000</ns0:v>
+      </ns0:c>
+      <ns0:c r="G4" s="8">
+        <ns0:f>MAX(0,E4-Perspectivas!$C$2)</ns0:f>
+        <ns0:v>24000</ns0:v>
+      </ns0:c>
+      <ns0:c r="H4" s="8">
+        <ns0:f>MAX(0,E4-Perspectivas!$D$2)</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I4" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>planning.json; mínimo financeiro sem reserva, receita e custos de implantação. Antes do desembolso, resolver financiamento. Nos demais marcos, caixa não comprova aceite; parar se faltar acesso, recursos ou segurança.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5" ht="120" customHeight="1">
+      <ns0:c r="A5" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Mês 3</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Medir qualidade e recuperar falhas</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C5" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Benchmark na DGX, fila e recusa, exportação, recuperação e fluxo de reunião. Orçamento mínimo M0–M3: R$211 mil, sem reserva.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D5" s="10">
+        <ns0:v>3</ns0:v>
+      </ns0:c>
+      <ns0:c r="E5" s="8">
+        <ns0:f>Perspectivas!$B$5+D5*Premissas!$B$10</ns0:f>
+        <ns0:v>211000</ns0:v>
+      </ns0:c>
+      <ns0:c r="F5" s="8">
+        <ns0:f>MAX(0,E5-Perspectivas!$B$2)</ns0:f>
+        <ns0:v>111000</ns0:v>
+      </ns0:c>
+      <ns0:c r="G5" s="8">
+        <ns0:f>MAX(0,E5-Perspectivas!$C$2)</ns0:f>
+        <ns0:v>61000</ns0:v>
+      </ns0:c>
+      <ns0:c r="H5" s="8">
+        <ns0:f>MAX(0,E5-Perspectivas!$D$2)</ns0:f>
+        <ns0:v>11000</ns0:v>
+      </ns0:c>
+      <ns0:c r="I5" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>planning.json; mínimo financeiro sem reserva, receita e custos de implantação. Antes do desembolso, resolver financiamento. Nos demais marcos, caixa não comprova aceite; parar se faltar acesso, recursos ou segurança.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6" ht="120" customHeight="1">
+      <ns0:c r="A6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Meses 4–6</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Homologar o recorte comercial</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Conectores suportados, segurança, limites contratuais e usuários de validação. Se faltarem recursos ou acesso, interromper avanço, não declarar entrega.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D6" s="10">
+        <ns0:v>6</ns0:v>
+      </ns0:c>
+      <ns0:c r="E6" s="8">
+        <ns0:f>Perspectivas!$B$5+D6*Premissas!$B$10</ns0:f>
+        <ns0:v>322000</ns0:v>
+      </ns0:c>
+      <ns0:c r="F6" s="8">
+        <ns0:f>MAX(0,E6-Perspectivas!$B$2)</ns0:f>
+        <ns0:v>222000</ns0:v>
+      </ns0:c>
+      <ns0:c r="G6" s="8">
+        <ns0:f>MAX(0,E6-Perspectivas!$C$2)</ns0:f>
+        <ns0:v>172000</ns0:v>
+      </ns0:c>
+      <ns0:c r="H6" s="8">
+        <ns0:f>MAX(0,E6-Perspectivas!$D$2)</ns0:f>
+        <ns0:v>122000</ns0:v>
+      </ns0:c>
+      <ns0:c r="I6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>planning.json; mínimo financeiro sem reserva, receita e custos de implantação. Antes do desembolso, resolver financiamento. Nos demais marcos, caixa não comprova aceite; parar se faltar acesso, recursos ou segurança.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7" ht="120" customHeight="1">
+      <ns0:c r="A7" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>A partir do mês 7 no cenário-base</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B7" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Entregar o primeiro ambiente pago</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C7" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Contrato e entrada recebida antes do início; três meses e 720 horas diretas separados do P&amp;D. Não é receita garantida.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D7" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Não estimado aqui</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E7" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Não estimado aqui</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F7" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Não estimado aqui</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G7" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Não estimado aqui</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H7" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Não estimado aqui</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I7" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>M7 é hipótese-base, não venda comprovada. Contrato + entrada recebida. Custos diretos e recebimentos têm calendário próprio no fluxo Base; não extrapolar R$37 mil/mês como custo total.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="10">
+      <ns0:c r="A10" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Implantação principal</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B10" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Horas diretas</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C10" s="10">
+        <ns0:f>Premissas!B4*(1+Premissas!B5)</ns0:f>
+        <ns0:v>720</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="11">
+      <ns0:c r="B11" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Custo direto por implantação</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C11" s="8">
+        <ns0:f>C10*Premissas!B6</ns0:f>
+        <ns0:v>129600</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="12" ht="90" customHeight="1">
+      <ns0:c r="B12" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Sequência de construção</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C12" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Núcleo e Topologic Operação primeiro. Diagnóstico valida comprador/recorte. Consulta privada após isolamento/carga; Viva após oferta repetível; parceiros após método e contratos. Não cinco produtos simultâneos.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="13" ht="90" customHeight="1">
+      <ns0:c r="B13" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Capacidade e privacidade</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C13" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Uma implantação por vez; P&amp;D separado. 100 usuários, 20 simultâneos no mapa, 1 IA ativa + 2 em fila: metas compartilhadas, não benchmark. Uma DGX sem redundância. Sem reutilizar dados de clientes entre ofertas.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ns0:pageSetup fitToHeight="0" orientation="landscape"/>
+</ns0:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetPr>
+    <ns0:pageSetUpPr fitToPage="1"/>
+  </ns0:sheetPr>
+  <ns0:dimension ref="A1:Q20"/>
+  <ns0:sheetFormatPr defaultRowHeight="15"/>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="29.7109375" customWidth="1"/>
+    <ns0:col min="2" max="3" width="22.7109375" customWidth="1"/>
+    <ns0:col min="4" max="4" width="16.7109375" customWidth="1"/>
+    <ns0:col min="5" max="6" width="20.7109375" customWidth="1"/>
+    <ns0:col min="7" max="8" width="15.7109375" customWidth="1"/>
+    <ns0:col min="9" max="12" width="22.7109375" customWidth="1"/>
+    <ns0:col min="13" max="13" width="48.7109375" customWidth="1"/>
+    <ns0:col min="14" max="14" width="85.7109375" customWidth="1"/>
+    <ns0:col min="15" max="15" width="65.7109375" customWidth="1"/>
+    <ns0:col min="16" max="16" width="90.7109375" customWidth="1"/>
+    <ns0:col min="17" max="17" width="65.7109375" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" ht="42" customHeight="1">
+      <ns0:c r="A1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Oferta</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Setup proposto</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Mensalidade proposta</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Horas setup</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Horas curadoria/mês</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Custo/hora</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Tributos</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Comercial</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Direto setup</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Direto/mês</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Contribuição setup</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Contribuição/mês</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Comprador</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Escopo</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Reuso compartilhado</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="P1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Pré-requisito</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="Q1" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Status / fonte</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2" ht="165" customHeight="1">
+      <ns0:c r="A2" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Diagnóstico operacional</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B2" s="8">
+        <ns0:v>30000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C2" s="8">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="D2" s="10">
+        <ns0:v>80</ns0:v>
+      </ns0:c>
+      <ns0:c r="E2" s="10">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="F2" s="8">
+        <ns0:f>Premissas!$B$6</ns0:f>
+        <ns0:v>180</ns0:v>
+      </ns0:c>
+      <ns0:c r="G2" s="11">
+        <ns0:f>Premissas!$B$8</ns0:f>
+        <ns0:v>0.12</ns0:v>
+      </ns0:c>
+      <ns0:c r="H2" s="11">
+        <ns0:f>Premissas!$B$9</ns0:f>
+        <ns0:v>0.05</ns0:v>
+      </ns0:c>
+      <ns0:c r="I2" s="8">
+        <ns0:f>D2*F2</ns0:f>
+        <ns0:v>14400</ns0:v>
+      </ns0:c>
+      <ns0:c r="J2" s="8">
+        <ns0:f>E2*F2</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="K2" s="8">
+        <ns0:f>B2*(1-G2-H2)-I2</ns0:f>
+        <ns0:v>10500</ns0:v>
+      </ns0:c>
+      <ns0:c r="L2" s="8">
+        <ns0:f>C2*(1-G2-H2)-J2</ns0:f>
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="M2" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Patrocinador de uma mudança industrial ou logística</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N2" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Um recorte, fontes autorizadas, mapa de dependências e perguntas de decisão; sem integração produtiva.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O2" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Método, editor e processamento documental em janela agendada</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="P2" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Validar disposição de pagar, acesso e escopo. Se o valor for creditado no setup, não somar as duas receitas integralmente.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="Q2" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Nova hipótese comercial; fora do fluxo de 24 meses; planning.json, hipóteses não validadas</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3" ht="165" customHeight="1">
+      <ns0:c r="A3" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Topologic Operação</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3" s="8">
+        <ns0:f>Premissas!B2</ns0:f>
+        <ns0:v>200000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C3" s="8">
+        <ns0:f>Premissas!B3</ns0:f>
+        <ns0:v>12000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D3" s="10">
+        <ns0:f>Premissas!B4*(1+Premissas!B5)</ns0:f>
+        <ns0:v>720</ns0:v>
+      </ns0:c>
+      <ns0:c r="E3" s="10">
+        <ns0:f>Premissas!B7</ns0:f>
+        <ns0:v>10</ns0:v>
+      </ns0:c>
+      <ns0:c r="F3" s="8">
+        <ns0:f>Premissas!$B$6</ns0:f>
+        <ns0:v>180</ns0:v>
+      </ns0:c>
+      <ns0:c r="G3" s="11">
+        <ns0:f>Premissas!$B$8</ns0:f>
+        <ns0:v>0.12</ns0:v>
+      </ns0:c>
+      <ns0:c r="H3" s="11">
+        <ns0:f>Premissas!$B$9</ns0:f>
+        <ns0:v>0.05</ns0:v>
+      </ns0:c>
+      <ns0:c r="I3" s="8">
+        <ns0:f>D3*F3</ns0:f>
+        <ns0:v>129600</ns0:v>
+      </ns0:c>
+      <ns0:c r="J3" s="8">
+        <ns0:f>E3*F3</ns0:f>
+        <ns0:v>1800</ns0:v>
+      </ns0:c>
+      <ns0:c r="K3" s="8">
+        <ns0:f>B3*(1-G3-H3)-I3</ns0:f>
+        <ns0:v>36400</ns0:v>
+      </ns0:c>
+      <ns0:c r="L3" s="8">
+        <ns0:f>C3*(1-G3-H3)-J3</ns0:f>
+        <ns0:v>8160</ns0:v>
+      </ns0:c>
+      <ns0:c r="M3" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Diretor de operações com transformação financiada</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N3" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Uma unidade, até três processos relacionados, dois conectores homologados, 150 entidades e dez usuários.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O3" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Grafo de conhecimento, fontes, permissões, visões e inferência</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="P3" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Produto e conectores homologados, contrato e entrada recebida. Oferta proposta, não vendas comprovadas.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="Q3" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Oferta principal; única linha nas projeções de 24 meses; planning.json, hipóteses não validadas</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4" ht="165" customHeight="1">
+      <ns0:c r="A4" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Conhecimento privado</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B4" s="8">
+        <ns0:v>60000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C4" s="8">
+        <ns0:v>6000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D4" s="10">
+        <ns0:v>180</ns0:v>
+      </ns0:c>
+      <ns0:c r="E4" s="10">
+        <ns0:v>6</ns0:v>
+      </ns0:c>
+      <ns0:c r="F4" s="8">
+        <ns0:f>Premissas!$B$6</ns0:f>
+        <ns0:v>180</ns0:v>
+      </ns0:c>
+      <ns0:c r="G4" s="11">
+        <ns0:f>Premissas!$B$8</ns0:f>
+        <ns0:v>0.12</ns0:v>
+      </ns0:c>
+      <ns0:c r="H4" s="11">
+        <ns0:f>Premissas!$B$9</ns0:f>
+        <ns0:v>0.05</ns0:v>
+      </ns0:c>
+      <ns0:c r="I4" s="8">
+        <ns0:f>D4*F4</ns0:f>
+        <ns0:v>32400</ns0:v>
+      </ns0:c>
+      <ns0:c r="J4" s="8">
+        <ns0:f>E4*F4</ns0:f>
+        <ns0:v>1080</ns0:v>
+      </ns0:c>
+      <ns0:c r="K4" s="8">
+        <ns0:f>B4*(1-G4-H4)-I4</ns0:f>
+        <ns0:v>17400</ns0:v>
+      </ns0:c>
+      <ns0:c r="L4" s="8">
+        <ns0:f>C4*(1-G4-H4)-J4</ns0:f>
+        <ns0:v>3900</ns0:v>
+      </ns0:c>
+      <ns0:c r="M4" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Área com documentação técnica e necessidade de consulta restrita</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N4" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Consulta documental com fontes e permissões, sem promessa de mapear toda a operação.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O4" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Ingestão, busca, identidade, armazenamento e IA local</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="P4" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Teste de isolamento, qualidade, retenção e carga. Limites de corpus e usuários definidos antes da proposta. Não é produto pronto.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="Q4" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Nova hipótese comercial; fora do fluxo de 24 meses; planning.json, hipóteses não validadas</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5" ht="165" customHeight="1">
+      <ns0:c r="A5" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Topologia Viva</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" s="8">
+        <ns0:v>90000</ns0:v>
+      </ns0:c>
+      <ns0:c r="C5" s="8">
+        <ns0:v>8000</ns0:v>
+      </ns0:c>
+      <ns0:c r="D5" s="10">
+        <ns0:v>300</ns0:v>
+      </ns0:c>
+      <ns0:c r="E5" s="10">
+        <ns0:v>8</ns0:v>
+      </ns0:c>
+      <ns0:c r="F5" s="8">
+        <ns0:f>Premissas!$B$6</ns0:f>
+        <ns0:v>180</ns0:v>
+      </ns0:c>
+      <ns0:c r="G5" s="11">
+        <ns0:f>Premissas!$B$8</ns0:f>
+        <ns0:v>0.12</ns0:v>
+      </ns0:c>
+      <ns0:c r="H5" s="11">
+        <ns0:f>Premissas!$B$9</ns0:f>
+        <ns0:v>0.05</ns0:v>
+      </ns0:c>
+      <ns0:c r="I5" s="8">
+        <ns0:f>D5*F5</ns0:f>
+        <ns0:v>54000</ns0:v>
+      </ns0:c>
+      <ns0:c r="J5" s="8">
+        <ns0:f>E5*F5</ns0:f>
+        <ns0:v>1440</ns0:v>
+      </ns0:c>
+      <ns0:c r="K5" s="8">
+        <ns0:f>B5*(1-G5-H5)-I5</ns0:f>
+        <ns0:v>20700</ns0:v>
+      </ns0:c>
+      <ns0:c r="L5" s="8">
+        <ns0:f>C5*(1-G5-H5)-J5</ns0:f>
+        <ns0:v>5200</ns0:v>
+      </ns0:c>
+      <ns0:c r="M5" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Cliente Topologic já homologado</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N5" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Um fluxo de observação e ação assistida, com aprovação humana e destinos autorizados.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O5" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Eventos, contexto do grafo, fila, auditoria e inferência</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="P5" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Somente após oferta principal repetível. Homologar integração, limites, parada e recuperação. Não vender autonomia irrestrita.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="Q5" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Expansão futura; fora do fluxo de 24 meses; planning.json, hipóteses não validadas</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6" ht="165" customHeight="1">
+      <ns0:c r="A6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Licenciamento com parceiros</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>A definir</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>A definir</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>A definir</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>A definir</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>A definir</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>A definir</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>A definir</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>A definir</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>A definir</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>A definir</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>A definir</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Integradores de indústria e logística</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Distribuição e implantação com método e componentes reutilizáveis, nunca revenda de dados de clientes.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Ontologias próprias, editor, conectores homologados e método</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="P6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Preço, direitos, suporte, responsabilidades e repartição de receita ainda precisam ser definidos. Não presumir comissão de 5% suficiente.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="Q6" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Canal posterior, sem receita precificada ou projetada; planning.json, hipóteses não validadas</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9" ht="175" customHeight="1">
+      <ns0:c r="A9" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Economia unitária</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B9" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Contribuição não é lucro. Comparação estável usa 12% + 5%; fluxo 24 meses separa faturamento e recebimentos. Custos fixos e capital não são abatidos nesta contribuição.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="10" ht="175" customHeight="1">
+      <ns0:c r="A10" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Sem receita adicional projetada</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B10" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Somente Topologic Operação está nas abas de 24 meses. Outras ofertas não reduzem déficits; canais e preços não comprovados. Parceiros sem preço ou margem calculável; 5% não é comissão negociada.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="11" ht="175" customHeight="1">
+      <ns0:c r="A11" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Recursos e sequência</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B11" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Mesma DGX, pessoas, fila, armazenamento e janelas. Não multiplicar capacidade por oferta nem contar P&amp;D como implantação. Núcleo primeiro; ofertas adjacentes dependem de homologação. Nenhum aluguel ilimitado de GPU.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="12" ht="175" customHeight="1">
+      <ns0:c r="A12" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Privacidade</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B12" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Reutilizar código, ontologias próprias e método; nunca dados de clientes. Isolamento, retenção, fontes autorizadas e LGPD por oferta; IA local não elimina risco de vazamento.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="14" ht="60" customHeight="1">
+      <ns0:c r="A14" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Crédito integral de diagnóstico no setup</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B14" s="8">
+        <ns0:f>B2</ns0:f>
+        <ns0:v>30000</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="15" ht="60" customHeight="1">
+      <ns0:c r="A15" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Saldo de setup após crédito</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B15" s="8">
+        <ns0:f>B3-B14</ns0:f>
+        <ns0:v>170000</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="16" ht="60" customHeight="1">
+      <ns0:c r="A16" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Receita combinada, sem duplicação</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B16" s="8">
+        <ns0:f>B2+B15</ns0:f>
+        <ns0:v>200000</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="17" ht="60" customHeight="1">
+      <ns0:c r="A17" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Diretos combinados: 80h adicionais às 720h</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B17" s="8">
+        <ns0:f>I2+I3</ns0:f>
+        <ns0:v>144000</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="18" ht="60" customHeight="1">
+      <ns0:c r="A18" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Contribuição combinada antes de fixos</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B18" s="8">
+        <ns0:f>B16*(1-G3-H3)-B17</ns0:f>
+        <ns0:v>22000</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="20" ht="200" customHeight="1">
+      <ns0:c r="A20" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hipótese do crédito</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B20" s="7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Exemplo conservador: diagnóstico 80h adicional às 720h. Crédito comercial não apaga custo. Se houver reuso comprovado, revisar escopo/horas sem duplicação. Não somar R$30 mil + R$200 mil de receita quando os R$30 mil são creditados.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ns0:pageSetup fitToHeight="0" orientation="landscape"/>
+</ns0:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>